<commit_message>
added output excel files
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2054,6 +2054,141 @@
         <v>63</v>
       </c>
     </row>
+    <row r="65">
+      <c r="A65" t="inlineStr"/>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>16</v>
+      </c>
+      <c r="D65" t="n">
+        <v>0</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>02/05/2025 08:50:16</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>20250502_9872.jpg</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr"/>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>16</v>
+      </c>
+      <c r="D66" t="n">
+        <v>0</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>02/05/2025 08:50:26</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>20250502_9459.jpg</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr"/>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>16</v>
+      </c>
+      <c r="D67" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>02/05/2025 08:50:37</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>20250502_5227.jpg</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr"/>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>16</v>
+      </c>
+      <c r="D68" t="n">
+        <v>0</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>02/05/2025 08:50:48</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>20250502_3912.jpg</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr"/>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>16</v>
+      </c>
+      <c r="D69" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>02/05/2025 08:50:59</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>20250502_2880.jpg</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>